<commit_message>
Add facility contact details
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sil-facility-import-template.xlsx
+++ b/frontend/public/templates/sil-facility-import-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cache\Shipment-Intelligence-Layer\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEFD1EB0-56DA-4E2E-89F1-5C5F20F2B0EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24C5E10-0CCE-4E73-9422-11C4581600BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" xr2:uid="{2FA0A343-03D9-488E-8EA9-3457B79D4D2B}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Facility Name</t>
   </si>
@@ -66,6 +66,21 @@
   </si>
   <si>
     <t>Site ID</t>
+  </si>
+  <si>
+    <t>Primary Contact Name</t>
+  </si>
+  <si>
+    <t>Primary Contact Title</t>
+  </si>
+  <si>
+    <t>Primary Contact Email</t>
+  </si>
+  <si>
+    <t>Primary Contact Phone</t>
+  </si>
+  <si>
+    <t>Operating Hours</t>
   </si>
 </sst>
 </file>
@@ -464,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A05E8E4-3183-41B8-AD6E-4166B1A20233}">
-  <dimension ref="A1:H501"/>
+  <dimension ref="A1:M501"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -474,9 +489,13 @@
     <col min="5" max="5" width="12.7109375" customWidth="1"/>
     <col min="6" max="6" width="14.7109375" customWidth="1"/>
     <col min="7" max="8" width="18.7109375" customWidth="1"/>
+    <col min="9" max="10" width="22.7109375" customWidth="1"/>
+    <col min="11" max="11" width="30.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -501,8 +520,23 @@
       <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -512,7 +546,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -522,7 +556,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -532,7 +566,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -542,7 +576,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -552,7 +586,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -562,7 +596,7 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -572,7 +606,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -582,7 +616,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -592,7 +626,7 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -602,7 +636,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -612,7 +646,7 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -622,7 +656,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -632,7 +666,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -642,7 +676,7 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -5503,7 +5537,6 @@
       <c r="H501" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{9A05E8E4-3183-41B8-AD6E-4166B1A20233}"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G501" xr:uid="{84D46FCF-CD5B-430D-BF96-45A9A138682E}">
       <formula1>"Supplier,Cross-dock,DC,MFC,Other"</formula1>

</xml_diff>

<commit_message>
Add facility ownership fields
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sil-facility-import-template.xlsx
+++ b/frontend/public/templates/sil-facility-import-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cache\Shipment-Intelligence-Layer\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24C5E10-0CCE-4E73-9422-11C4581600BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9024F21-BD44-4A13-B9B6-CC0148F9B039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" xr2:uid="{2FA0A343-03D9-488E-8EA9-3457B79D4D2B}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Facility Name</t>
   </si>
@@ -81,6 +81,12 @@
   </si>
   <si>
     <t>Operating Hours</t>
+  </si>
+  <si>
+    <t>Regional Manager</t>
+  </si>
+  <si>
+    <t>Supply Chain Business Partner</t>
   </si>
 </sst>
 </file>
@@ -479,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A05E8E4-3183-41B8-AD6E-4166B1A20233}">
-  <dimension ref="A1:M501"/>
+  <dimension ref="A1:O501"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
@@ -492,10 +498,11 @@
     <col min="9" max="10" width="22.7109375" customWidth="1"/>
     <col min="11" max="11" width="30.7109375" customWidth="1"/>
     <col min="12" max="12" width="22.7109375" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" customWidth="1"/>
+    <col min="13" max="14" width="24.7109375" customWidth="1"/>
+    <col min="15" max="15" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -535,8 +542,14 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -546,7 +559,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -556,7 +569,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -566,7 +579,7 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -576,7 +589,7 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -586,7 +599,7 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -596,7 +609,7 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -606,7 +619,7 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -616,7 +629,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -626,7 +639,7 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -636,7 +649,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -646,7 +659,7 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -656,7 +669,7 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -666,7 +679,7 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -676,7 +689,7 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>

</xml_diff>